<commit_message>
Add DROPPED status support for properties and fix property overview count
</commit_message>
<xml_diff>
--- a/uploads/M3M  CALLING DATA 1-381.xlsx
+++ b/uploads/M3M  CALLING DATA 1-381.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gaurav\Desktop\"/>
     </mc:Choice>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="1039">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1146" uniqueCount="1040">
   <si>
     <t>ASHISH MITTAL</t>
   </si>
@@ -3153,12 +3153,16 @@
   </si>
   <si>
     <t>REMARK1</t>
+  </si>
+  <si>
+    <t>NOT AVAILABEL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -3580,11 +3584,11 @@
   <dimension ref="A1:E382"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="52.7109375" customWidth="1"/>
-    <col min="2" max="2" width="27.140625" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" customWidth="1"/>
-    <col min="5" max="5" width="26.28515625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="52.7109375"/>
+    <col min="2" max="2" customWidth="true" width="27.140625"/>
+    <col min="3" max="3" customWidth="true" width="19.7109375"/>
+    <col min="4" max="4" customWidth="true" width="11.85546875"/>
+    <col min="5" max="5" customWidth="true" width="26.28515625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
@@ -4230,7 +4234,9 @@
       <c r="D43" s="1">
         <v>1021</v>
       </c>
-      <c r="E43" s="3"/>
+      <c r="E43" s="3" t="s">
+        <v>1039</v>
+      </c>
     </row>
     <row r="44" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">

</xml_diff>

<commit_message>
Fix: Facebook/Instagram source mapping and timezone configuration
- Add FACEBOOK and INSTAGRAM source mapping in WebhookController
- Fix notification messages for direct assignment leads
- Configure application timezone to Asia/Kolkata (IST)
- Update database timezone from UTC to Asia/Kolkata
- Add TimezoneConfig for global timezone setting
</commit_message>
<xml_diff>
--- a/uploads/M3M  CALLING DATA 1-381.xlsx
+++ b/uploads/M3M  CALLING DATA 1-381.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1146" uniqueCount="1040">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="1041">
   <si>
     <t>ASHISH MITTAL</t>
   </si>
@@ -3156,6 +3156,9 @@
   </si>
   <si>
     <t>NOT AVAILABEL</t>
+  </si>
+  <si>
+    <t>INCOMING CALL NOT AVAILABELL</t>
   </si>
 </sst>
 </file>
@@ -4296,7 +4299,9 @@
       <c r="D47" s="1">
         <v>1147.1199999999999</v>
       </c>
-      <c r="E47" s="3"/>
+      <c r="E47" s="3" t="s">
+        <v>1040</v>
+      </c>
     </row>
     <row r="48" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">

</xml_diff>